<commit_message>
docs: update presentation and team roster; remove temp office file
</commit_message>
<xml_diff>
--- a/docs/Team_Members.xlsx
+++ b/docs/Team_Members.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Healthcare-RAG-Powered-Medical-QA-Assistant\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EEA8BB1-89BE-4095-B1A6-0CEA22FA0C83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A77015D1-4499-4EE5-84E0-E897AB5C0004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Name</t>
   </si>
@@ -60,10 +60,25 @@
     <t>youssefgeorge989@gmail.com</t>
   </si>
   <si>
-    <t>kdoha37@gmail.com</t>
-  </si>
-  <si>
-    <t>Eman.elkalawy018@gmail.com</t>
+    <t>01125016702</t>
+  </si>
+  <si>
+    <t>01013223173</t>
+  </si>
+  <si>
+    <t>01274135641</t>
+  </si>
+  <si>
+    <t>01097633885</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01155542571 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">kdoha37@gmail.com </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eman.elkalawy018@gmail.com </t>
   </si>
 </sst>
 </file>
@@ -86,10 +101,12 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="8.5"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -149,10 +166,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -163,20 +181,100 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8.5"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FFAAAAAA"/>
+        </left>
+        <right/>
+        <top/>
+        <bottom style="medium">
+          <color rgb="FFAAAAAA"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8.5"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFAAAAAA"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFAAAAAA"/>
+        </right>
+        <top/>
+        <bottom style="medium">
+          <color rgb="FFAAAAAA"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -187,6 +285,18 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F1EFB988-8BE9-43FA-A065-8F4AA804384D}" name="Table1" displayName="Table1" ref="A1:C6" totalsRowShown="0">
+  <autoFilter ref="A1:C6" xr:uid="{F1EFB988-8BE9-43FA-A065-8F4AA804384D}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{CEBCF1AA-DB89-4F34-9DC9-C592EB0F813D}" name="Name" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{39335B55-77B3-4C79-8F50-C3CCE09F2D76}" name="Email" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{EB1F528F-55FC-4AE0-8643-6BA645B02B6F}" name="Phone Number" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -455,8 +565,9 @@
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.21875" customWidth="1"/>
+    <col min="2" max="2" width="30.77734375" customWidth="1"/>
+    <col min="3" max="3" width="16.109375" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -466,55 +577,77 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C2">
-        <v>1125016702</v>
+      <c r="C2" s="4" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="33" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>9</v>
       </c>
+      <c r="C3" s="4" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" ht="33" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>10</v>
       </c>
+      <c r="C4" s="4" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="5" spans="1:3" ht="33" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>11</v>
+        <v>16</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="33" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>12</v>
+        <v>17</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B3" r:id="rId1" xr:uid="{C52FE4A9-16FC-4798-A60E-8FA006DF70E9}"/>
+    <hyperlink ref="B4" r:id="rId2" xr:uid="{F9155637-4B9E-4F03-A4F7-ACF77C73C71B}"/>
+    <hyperlink ref="B5" r:id="rId3" xr:uid="{7129205C-19FD-4D9F-AF77-BE29FB8FCC47}"/>
+    <hyperlink ref="B6" r:id="rId4" xr:uid="{79D3C397-9BE2-487F-BAB9-A3F5859FFE57}"/>
+    <hyperlink ref="B2" r:id="rId5" xr:uid="{A346A838-CD6E-4673-A747-FB9C89093BB6}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId6"/>
+  <tableParts count="1">
+    <tablePart r:id="rId7"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>